<commit_message>
Align MoC workbook with Sam's MOC Proposal Rev2 (stage requirements)
Replacement in Kind becomes Simple Change, Priority kept, Sam's captions
(Change Type, Change Impact, Change Justification, Approval Notes,
Lessons Learnt), per-stage mandatory flags and conditional justification
fields, task 'Required Before'. Every change tagged with its source.
Screening data load and question list updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - MOC Screening Questions - Data Load Draft.xlsx
+++ b/docs/moc/Impala - MOC Screening Questions - Data Load Draft.xlsx
@@ -134,9 +134,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScreeningQuestions" displayName="ScreeningQuestions" ref="A1:K80" headerRowCount="1">
-  <autoFilter ref="A1:K80"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScreeningQuestions" displayName="ScreeningQuestions" ref="A1:L80" headerRowCount="1">
+  <autoFilter ref="A1:L80"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Item Number"/>
     <tableColumn id="2" name="Checklist Item"/>
     <tableColumn id="3" name="Category"/>
@@ -144,10 +144,11 @@
     <tableColumn id="5" name="WF Stages"/>
     <tableColumn id="6" name="Change Impacts (blank = all)"/>
     <tableColumn id="7" name="Emergency Change? (blank = always)"/>
-    <tableColumn id="8" name="Temporary Change? (blank = always)"/>
-    <tableColumn id="9" name="MOC Categories (blank = all)"/>
-    <tableColumn id="10" name="Locations"/>
-    <tableColumn id="11" name="Impala Remarks"/>
+    <tableColumn id="8" name="Simple Change? (No = not generated for Simple Changes)"/>
+    <tableColumn id="9" name="Temporary Change? (blank = always)"/>
+    <tableColumn id="10" name="MOC Categories (blank = all)"/>
+    <tableColumn id="11" name="Locations"/>
+    <tableColumn id="12" name="Impala Remarks"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -442,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -461,47 +462,54 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Source: 'MOC Proposal.xlsx' &gt; 'Evaluation, D&amp;A Checklist' (Sam Robinson, draft under review).</t>
+          <t>Source: 'MOC Proposal Rev2.xlsx' &gt; 'Evaluation, D&amp;A Checklist' (Sam Robinson, under team review; unchanged vs Rev1).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Columns follow the Intelex 'MOC Screening Question Setup' object (workbook Fields rows 279-293).</t>
+          <t>Sam Rev2: checklist answered in Evaluation, Design &amp; Analysis (view-only later), is a MINIMUM (users may add items) and is NOT generated for Simple Changes (Simple Change? = No).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Part 1 (Universal) attached to the top location; Part 2 to the Liquids segment node; Part 3 to the Dry segment node.</t>
+          <t>Columns follow the Intelex 'MOC Screening Question Setup' object (workbook Fields rows 279-293).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Second 'J.' section in the source (Pre-Start-Up &amp; Close-Out) renumbered as 'K.'; its items go to Start Up / Follow Up.</t>
+          <t>Part 1 (Universal) attached to the top location; Part 2 to the Liquids segment node; Part 3 to the Dry segment node.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Blank filter = question generated regardless of that parameter (Intelex setup behaviour).</t>
+          <t>Second 'J.' section in the source (Pre-Start-Up &amp; Close-Out) renumbered as 'K.' (planned in EDA; verified by the Implementation / Follow Up questions).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>OPEN [TBC]: reduce the question set by Grade of Change (Minor short list / Major full list); answers Yes / No / N/A.</t>
+          <t>Blank filter = question generated regardless of that parameter (Intelex setup behaviour).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>OPEN [TBC]: link items to Change Type / Change Impact (e.g. HAZOP mandatory for Major equipment change); answers Yes / No / N/A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Intelex to confirm import template format before loading.</t>
         </is>
@@ -518,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K80"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -528,10 +536,11 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,20 +581,25 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Simple Change? (No = not generated for Simple Changes)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Temporary Change? (blank = always)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>MOC Categories (blank = all)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Locations</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Impala Remarks</t>
         </is>
@@ -617,14 +631,19 @@
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -652,14 +671,19 @@
       </c>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -687,14 +711,19 @@
       </c>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -722,14 +751,19 @@
       </c>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -757,14 +791,19 @@
       </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -792,14 +831,19 @@
       </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -831,14 +875,19 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Source note: 'Mandatory for Level 3+,' -&gt; mapped to Moderate/Major [TBC]</t>
         </is>
@@ -870,14 +919,19 @@
       </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -905,14 +959,19 @@
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -940,14 +999,19 @@
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -975,14 +1039,19 @@
       </c>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1010,14 +1079,19 @@
       </c>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1045,14 +1119,19 @@
       </c>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1080,14 +1159,19 @@
       </c>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1115,14 +1199,19 @@
       </c>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1150,14 +1239,19 @@
       </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1185,14 +1279,19 @@
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1220,14 +1319,19 @@
       </c>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1255,14 +1359,19 @@
       </c>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1290,14 +1399,19 @@
       </c>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1325,14 +1439,19 @@
       </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1360,14 +1479,19 @@
       </c>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1395,14 +1519,19 @@
       </c>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1430,14 +1559,19 @@
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1465,14 +1599,19 @@
       </c>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1500,14 +1639,19 @@
       </c>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1535,14 +1679,19 @@
       </c>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1570,14 +1719,19 @@
       </c>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1605,14 +1759,19 @@
       </c>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1640,14 +1799,19 @@
       </c>
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1675,14 +1839,19 @@
       </c>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1710,14 +1879,19 @@
       </c>
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1745,14 +1919,19 @@
       </c>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1780,14 +1959,19 @@
       </c>
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1815,14 +1999,19 @@
       </c>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1850,14 +2039,19 @@
       </c>
       <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1885,14 +2079,19 @@
       </c>
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1920,14 +2119,19 @@
       </c>
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1955,14 +2159,19 @@
       </c>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1990,14 +2199,19 @@
       </c>
       <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2025,14 +2239,19 @@
       </c>
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2060,14 +2279,19 @@
       </c>
       <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2095,14 +2319,19 @@
       </c>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2130,14 +2359,19 @@
       </c>
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2165,14 +2399,19 @@
       </c>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2200,14 +2439,19 @@
       </c>
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2235,14 +2479,19 @@
       </c>
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2270,14 +2519,19 @@
       </c>
       <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I49" s="2" t="inlineStr"/>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2305,14 +2559,19 @@
       </c>
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2340,14 +2599,19 @@
       </c>
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2375,14 +2639,19 @@
       </c>
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2410,14 +2679,19 @@
       </c>
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2445,14 +2719,19 @@
       </c>
       <c r="F54" s="2" t="inlineStr"/>
       <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2480,14 +2759,19 @@
       </c>
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2515,14 +2799,19 @@
       </c>
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2550,14 +2839,19 @@
       </c>
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2585,14 +2879,19 @@
       </c>
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -2620,14 +2919,19 @@
       </c>
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -2655,14 +2959,19 @@
       </c>
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -2690,14 +2999,19 @@
       </c>
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2725,14 +3039,19 @@
       </c>
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -2760,18 +3079,23 @@
       </c>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr"/>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
         <is>
           <t>4. Change of Control Systems / IT / SIS</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -2799,18 +3123,23 @@
       </c>
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
         <is>
           <t>4. Change of Control Systems / IT / SIS</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -2833,19 +3162,24 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Start Up</t>
+          <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr"/>
-      <c r="H65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -2868,19 +3202,24 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Follow Up</t>
+          <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -2903,23 +3242,28 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Follow Up</t>
+          <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr"/>
       <c r="G67" s="2" t="inlineStr"/>
       <c r="H67" s="2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -2942,19 +3286,24 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Follow Up</t>
+          <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr"/>
       <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr">
-        <is>
-          <t>Impala (top level - all terminals)</t>
-        </is>
-      </c>
-      <c r="K68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Impala (top level - all terminals)</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -2982,14 +3331,19 @@
       </c>
       <c r="F69" s="2" t="inlineStr"/>
       <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr">
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3017,14 +3371,19 @@
       </c>
       <c r="F70" s="2" t="inlineStr"/>
       <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr">
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3052,14 +3411,19 @@
       </c>
       <c r="F71" s="2" t="inlineStr"/>
       <c r="G71" s="2" t="inlineStr"/>
-      <c r="H71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr">
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -3087,14 +3451,19 @@
       </c>
       <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I72" s="2" t="inlineStr"/>
-      <c r="J72" s="2" t="inlineStr">
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3122,14 +3491,19 @@
       </c>
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I73" s="2" t="inlineStr"/>
-      <c r="J73" s="2" t="inlineStr">
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3157,14 +3531,19 @@
       </c>
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I74" s="2" t="inlineStr"/>
-      <c r="J74" s="2" t="inlineStr">
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3192,14 +3571,19 @@
       </c>
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I75" s="2" t="inlineStr"/>
-      <c r="J75" s="2" t="inlineStr">
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3227,14 +3611,19 @@
       </c>
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr"/>
-      <c r="H76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr">
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -3262,14 +3651,19 @@
       </c>
       <c r="F77" s="2" t="inlineStr"/>
       <c r="G77" s="2" t="inlineStr"/>
-      <c r="H77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I77" s="2" t="inlineStr"/>
-      <c r="J77" s="2" t="inlineStr">
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
         <is>
           <t>Liquids (business segment)</t>
         </is>
       </c>
-      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -3297,14 +3691,19 @@
       </c>
       <c r="F78" s="2" t="inlineStr"/>
       <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr">
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
         <is>
           <t>Dry (business segment)</t>
         </is>
       </c>
-      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -3332,14 +3731,19 @@
       </c>
       <c r="F79" s="2" t="inlineStr"/>
       <c r="G79" s="2" t="inlineStr"/>
-      <c r="H79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I79" s="2" t="inlineStr"/>
-      <c r="J79" s="2" t="inlineStr">
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr">
         <is>
           <t>Dry (business segment)</t>
         </is>
       </c>
-      <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3367,14 +3771,19 @@
       </c>
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr"/>
-      <c r="H80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="I80" s="2" t="inlineStr"/>
-      <c r="J80" s="2" t="inlineStr">
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
         <is>
           <t>Dry (business segment)</t>
         </is>
       </c>
-      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>